<commit_message>
Update Finance Vietcap: cập nhật quý tài chính mới 2026-07-17 02:56:10
</commit_message>
<xml_diff>
--- a/Output/sector_finance_ticker_data.xlsx
+++ b/Output/sector_finance_ticker_data.xlsx
@@ -7391,7 +7391,9 @@
       <c r="Z84" t="n">
         <v>1821305420483</v>
       </c>
-      <c r="AA84" t="inlineStr"/>
+      <c r="AA84" t="n">
+        <v>2016139061540</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
@@ -10819,7 +10821,9 @@
       <c r="Z126" t="n">
         <v>1185722562041</v>
       </c>
-      <c r="AA126" t="inlineStr"/>
+      <c r="AA126" t="n">
+        <v>1197467746023</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
@@ -21673,7 +21677,9 @@
       <c r="Z258" t="n">
         <v>2227394721247</v>
       </c>
-      <c r="AA258" t="inlineStr"/>
+      <c r="AA258" t="n">
+        <v>2241761026928</v>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="1" t="inlineStr">
@@ -31982,7 +31988,9 @@
       <c r="Z84" t="n">
         <v>-157486049561</v>
       </c>
-      <c r="AA84" t="inlineStr"/>
+      <c r="AA84" t="n">
+        <v>194833641057</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="1" t="inlineStr">
@@ -35410,7 +35418,9 @@
       <c r="Z126" t="n">
         <v>10916610256</v>
       </c>
-      <c r="AA126" t="inlineStr"/>
+      <c r="AA126" t="n">
+        <v>11745183982</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="1" t="inlineStr">
@@ -46229,7 +46239,9 @@
       <c r="Z257" t="n">
         <v>99719488125</v>
       </c>
-      <c r="AA257" t="inlineStr"/>
+      <c r="AA257" t="n">
+        <v>42044185666</v>
+      </c>
     </row>
     <row r="258">
       <c r="A258" s="1" t="inlineStr">

</xml_diff>